<commit_message>
Add Scott Alexander, Devin Bell, and Maddox Molony to the pro tracker.
Scott is Omaha/Royals, Devin is Ontario/Dodgers, and Maddox is Lakeland/Tigers; Bell and Molony come off the amateur list.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/client_lists/Client List - 04-15-26.xlsx
+++ b/client_lists/Client List - 04-15-26.xlsx
@@ -475,7 +475,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr autoPageBreaks="0"/>
   </sheetPr>
-  <dimension ref="A1:G118"/>
+  <dimension ref="A1:G120"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="24.6640625" customWidth="1" style="4" min="1" max="1"/>
@@ -811,32 +811,32 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="3" t="inlineStr">
-        <is>
-          <t>Bertrand, John Michael</t>
-        </is>
-      </c>
-      <c r="B12" s="3" t="inlineStr">
-        <is>
-          <t>Giants</t>
-        </is>
-      </c>
-      <c r="C12" s="3" t="inlineStr">
-        <is>
-          <t>Triple-A Pacific Coast League</t>
-        </is>
-      </c>
-      <c r="D12" s="3" t="inlineStr">
-        <is>
-          <t>Sacramento River Cats</t>
-        </is>
-      </c>
-      <c r="E12" s="3" t="inlineStr">
-        <is>
-          <t>LHP</t>
-        </is>
-      </c>
-      <c r="F12" s="3" t="inlineStr">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Bell, Devin</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Dodgers</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Single-A California League</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Ontario Tower Buzzers</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>RHP</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
         <is>
           <t>AK</t>
         </is>
@@ -845,22 +845,27 @@
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>Brogdon, Connor</t>
+          <t>Bertrand, John Michael</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>Guardians</t>
+          <t>Giants</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>Major Leagues</t>
+          <t>Triple-A Pacific Coast League</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>Sacramento River Cats</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>RHP</t>
+          <t>LHP</t>
         </is>
       </c>
       <c r="F13" s="3" t="inlineStr">
@@ -872,22 +877,17 @@
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>Brooks, Steven</t>
+          <t>Brogdon, Connor</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>Red Sox</t>
+          <t>Guardians</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>High-A South Atlantic League</t>
-        </is>
-      </c>
-      <c r="D14" s="3" t="inlineStr">
-        <is>
-          <t>Greenville Drive</t>
+          <t>Major Leagues</t>
         </is>
       </c>
       <c r="E14" s="3" t="inlineStr">
@@ -897,29 +897,29 @@
       </c>
       <c r="F14" s="3" t="inlineStr">
         <is>
-          <t>TJ</t>
+          <t>AK</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>Brown, Ryan</t>
+          <t>Brooks, Steven</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>Dodgers</t>
+          <t>Red Sox</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>R Arizona Complex League</t>
+          <t>High-A South Atlantic League</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>ACL Dodgers</t>
+          <t>Greenville Drive</t>
         </is>
       </c>
       <c r="E15" s="3" t="inlineStr">
@@ -929,88 +929,93 @@
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>JF</t>
+          <t>TJ</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>Bubic, Kris</t>
+          <t>Brown, Ryan</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>Royals</t>
+          <t>Dodgers</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>Major Leagues</t>
+          <t>R Arizona Complex League</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>ACL Dodgers</t>
         </is>
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>LHP</t>
+          <t>RHP</t>
         </is>
       </c>
       <c r="F16" s="3" t="inlineStr">
         <is>
-          <t>AK</t>
+          <t>JF</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>Burdi, Nick</t>
+          <t>Bubic, Kris</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>Mets</t>
+          <t>Royals</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>Triple-A International League</t>
-        </is>
-      </c>
-      <c r="D17" s="3" t="inlineStr">
-        <is>
-          <t>Syracuse Mets</t>
+          <t>Major Leagues</t>
         </is>
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>RHP</t>
+          <t>LHP</t>
         </is>
       </c>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>JF</t>
+          <t>AK</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>Burke, Brock</t>
+          <t>Burdi, Nick</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>Reds</t>
+          <t>Mets</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>Major Leagues</t>
+          <t>Triple-A International League</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>Syracuse Mets</t>
         </is>
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>LHP</t>
+          <t>RHP</t>
         </is>
       </c>
       <c r="F18" s="3" t="inlineStr">
@@ -1022,22 +1027,17 @@
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>Bush, Ky</t>
+          <t>Burke, Brock</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>White Sox</t>
+          <t>Reds</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>R Arizona Complex League</t>
-        </is>
-      </c>
-      <c r="D19" s="3" t="inlineStr">
-        <is>
-          <t>ACL White Sox</t>
+          <t>Major Leagues</t>
         </is>
       </c>
       <c r="E19" s="3" t="inlineStr">
@@ -1047,34 +1047,34 @@
       </c>
       <c r="F19" s="3" t="inlineStr">
         <is>
-          <t>AK</t>
+          <t>JF</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>Darby, Zander</t>
+          <t>Bush, Ky</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>Giants</t>
+          <t>White Sox</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>High-A Northwest League</t>
+          <t>R Arizona Complex League</t>
         </is>
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>Eugene Emeralds</t>
+          <t>ACL White Sox</t>
         </is>
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t>3B</t>
+          <t>LHP</t>
         </is>
       </c>
       <c r="F20" s="3" t="inlineStr">
@@ -1086,27 +1086,27 @@
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>Diaz, Davis</t>
+          <t>Darby, Zander</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>Athletics</t>
+          <t>Giants</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>High-A Midwest League</t>
+          <t>High-A Northwest League</t>
         </is>
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t>Lansing Lugnuts</t>
+          <t>Eugene Emeralds</t>
         </is>
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>3B</t>
         </is>
       </c>
       <c r="F21" s="3" t="inlineStr">
@@ -1118,22 +1118,27 @@
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>Dreyer, Jack</t>
+          <t>Diaz, Davis</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>Dodgers</t>
+          <t>Athletics</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>Major Leagues</t>
+          <t>High-A Midwest League</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>Lansing Lugnuts</t>
         </is>
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>LHP</t>
+          <t>C</t>
         </is>
       </c>
       <c r="F22" s="3" t="inlineStr">
@@ -1145,12 +1150,12 @@
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>Erceg, Lucas</t>
+          <t>Dreyer, Jack</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>Royals</t>
+          <t>Dodgers</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
@@ -1160,7 +1165,7 @@
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>RHP</t>
+          <t>LHP</t>
         </is>
       </c>
       <c r="F23" s="3" t="inlineStr">
@@ -1172,12 +1177,12 @@
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
-          <t>Fitzgerald, Tyler</t>
+          <t>Erceg, Lucas</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>Blue Jays</t>
+          <t>Royals</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
@@ -1187,93 +1192,93 @@
       </c>
       <c r="E24" s="3" t="inlineStr">
         <is>
-          <t>INF / OF</t>
+          <t>RHP</t>
         </is>
       </c>
       <c r="F24" s="3" t="inlineStr">
         <is>
-          <t>JF</t>
+          <t>AK</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
         <is>
-          <t>Ford, Walter</t>
+          <t>Fitzgerald, Tyler</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>Mariners</t>
+          <t>Blue Jays</t>
         </is>
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>High-A Northwest League</t>
-        </is>
-      </c>
-      <c r="D25" s="3" t="inlineStr">
-        <is>
-          <t>Everett AquaSox</t>
+          <t>Major Leagues</t>
         </is>
       </c>
       <c r="E25" s="3" t="inlineStr">
         <is>
-          <t>RHP</t>
+          <t>INF / OF</t>
         </is>
       </c>
       <c r="F25" s="3" t="inlineStr">
         <is>
-          <t>TJ</t>
+          <t>JF</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
         <is>
-          <t>Fraizer, Matt</t>
+          <t>Ford, Walter</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>Red Sox</t>
+          <t>Mariners</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>Triple-A International League</t>
+          <t>High-A Northwest League</t>
         </is>
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>Worcester Red Sox</t>
+          <t>Everett AquaSox</t>
         </is>
       </c>
       <c r="E26" s="3" t="inlineStr">
         <is>
-          <t>OF</t>
+          <t>RHP</t>
         </is>
       </c>
       <c r="F26" s="3" t="inlineStr">
         <is>
-          <t>AK</t>
+          <t>TJ</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
         <is>
-          <t>Friedl, TJ</t>
+          <t>Fraizer, Matt</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>Reds</t>
+          <t>Red Sox</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>Major Leagues</t>
+          <t>Triple-A International League</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>Worcester Red Sox</t>
         </is>
       </c>
       <c r="E27" s="3" t="inlineStr">
@@ -1290,27 +1295,22 @@
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
         <is>
-          <t>Gallagher, Ryan</t>
+          <t>Friedl, TJ</t>
         </is>
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>Twins</t>
+          <t>Reds</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>Double-A Texas League</t>
-        </is>
-      </c>
-      <c r="D28" s="3" t="inlineStr">
-        <is>
-          <t>Wichita Wind Surge</t>
+          <t>Major Leagues</t>
         </is>
       </c>
       <c r="E28" s="3" t="inlineStr">
         <is>
-          <t>RHP</t>
+          <t>OF</t>
         </is>
       </c>
       <c r="F28" s="3" t="inlineStr">
@@ -1322,54 +1322,54 @@
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
         <is>
-          <t>Gladney, DJ</t>
+          <t>Gallagher, Ryan</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>Yankees</t>
+          <t>Twins</t>
         </is>
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>Double-A Eastern League</t>
+          <t>Double-A Texas League</t>
         </is>
       </c>
       <c r="D29" s="3" t="inlineStr">
         <is>
-          <t>Somerset Patriots</t>
+          <t>Wichita Wind Surge</t>
         </is>
       </c>
       <c r="E29" s="3" t="inlineStr">
         <is>
-          <t>OF</t>
+          <t>RHP</t>
         </is>
       </c>
       <c r="F29" s="3" t="inlineStr">
         <is>
-          <t>TJ</t>
+          <t>AK</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
         <is>
-          <t>Glasser, Phillip</t>
+          <t>Gladney, DJ</t>
         </is>
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>Nationals</t>
+          <t>Yankees</t>
         </is>
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>Triple-A International League</t>
+          <t>Double-A Eastern League</t>
         </is>
       </c>
       <c r="D30" s="3" t="inlineStr">
         <is>
-          <t>Rochester Red Wings</t>
+          <t>Somerset Patriots</t>
         </is>
       </c>
       <c r="E30" s="3" t="inlineStr">
@@ -1379,34 +1379,34 @@
       </c>
       <c r="F30" s="3" t="inlineStr">
         <is>
-          <t>JF</t>
+          <t>TJ</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
         <is>
-          <t>Gray, Drew</t>
+          <t>Glasser, Phillip</t>
         </is>
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>Cubs</t>
+          <t>Nationals</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>R Arizona Complex League</t>
+          <t>Triple-A International League</t>
         </is>
       </c>
       <c r="D31" s="3" t="inlineStr">
         <is>
-          <t>ACL Cubs</t>
+          <t>Rochester Red Wings</t>
         </is>
       </c>
       <c r="E31" s="3" t="inlineStr">
         <is>
-          <t>LHP</t>
+          <t>OF</t>
         </is>
       </c>
       <c r="F31" s="3" t="inlineStr">
@@ -1418,49 +1418,54 @@
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
         <is>
-          <t>Green, Rodney</t>
+          <t>Gray, Drew</t>
         </is>
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>Athletics</t>
+          <t>Cubs</t>
         </is>
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>High-A Midwest League</t>
+          <t>R Arizona Complex League</t>
         </is>
       </c>
       <c r="D32" s="3" t="inlineStr">
         <is>
-          <t>Lansing Lugnuts</t>
+          <t>ACL Cubs</t>
         </is>
       </c>
       <c r="E32" s="3" t="inlineStr">
         <is>
-          <t>OF</t>
+          <t>LHP</t>
         </is>
       </c>
       <c r="F32" s="3" t="inlineStr">
         <is>
-          <t>AK</t>
+          <t>JF</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
         <is>
-          <t>Greene, Riley</t>
+          <t>Green, Rodney</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>Tigers</t>
+          <t>Athletics</t>
         </is>
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>Major Leagues</t>
+          <t>High-A Midwest League</t>
+        </is>
+      </c>
+      <c r="D33" s="3" t="inlineStr">
+        <is>
+          <t>Lansing Lugnuts</t>
         </is>
       </c>
       <c r="E33" s="3" t="inlineStr">
@@ -1470,29 +1475,24 @@
       </c>
       <c r="F33" s="3" t="inlineStr">
         <is>
-          <t>TJ</t>
+          <t>AK</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
         <is>
-          <t>Halpin, Petey</t>
+          <t>Greene, Riley</t>
         </is>
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>Guardians</t>
+          <t>Tigers</t>
         </is>
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>Triple-A International League</t>
-        </is>
-      </c>
-      <c r="D34" s="3" t="inlineStr">
-        <is>
-          <t>Columbus Clippers</t>
+          <t>Major Leagues</t>
         </is>
       </c>
       <c r="E34" s="3" t="inlineStr">
@@ -1502,153 +1502,157 @@
       </c>
       <c r="F34" s="3" t="inlineStr">
         <is>
-          <t>AK</t>
+          <t>TJ</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
         <is>
+          <t>Halpin, Petey</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="inlineStr">
+        <is>
+          <t>Guardians</t>
+        </is>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>Triple-A International League</t>
+        </is>
+      </c>
+      <c r="D35" s="3" t="inlineStr">
+        <is>
+          <t>Columbus Clippers</t>
+        </is>
+      </c>
+      <c r="E35" s="3" t="inlineStr">
+        <is>
+          <t>OF</t>
+        </is>
+      </c>
+      <c r="F35" s="3" t="inlineStr">
+        <is>
+          <t>AK</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="3" t="inlineStr">
+        <is>
           <t>Harvey, Ryan</t>
         </is>
       </c>
-      <c r="B35" s="3" t="inlineStr">
+      <c r="B36" s="3" t="inlineStr">
         <is>
           <t>Tigers</t>
         </is>
       </c>
-      <c r="C35" s="3" t="inlineStr">
+      <c r="C36" s="3" t="inlineStr">
         <is>
           <t>High-A Midwest League</t>
         </is>
       </c>
-      <c r="D35" s="3" t="inlineStr">
+      <c r="D36" s="3" t="inlineStr">
         <is>
           <t>West Michigan Whitecaps</t>
         </is>
       </c>
-      <c r="E35" s="3" t="inlineStr">
-        <is>
-          <t>RHP</t>
-        </is>
-      </c>
-      <c r="F35" s="3" t="inlineStr">
-        <is>
-          <t>AK</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
+      <c r="E36" s="3" t="inlineStr">
+        <is>
+          <t>RHP</t>
+        </is>
+      </c>
+      <c r="F36" s="3" t="inlineStr">
+        <is>
+          <t>AK</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
         <is>
           <t>Helfrick, Ryder</t>
         </is>
       </c>
-      <c r="B36" t="inlineStr">
+      <c r="B37" t="inlineStr">
         <is>
           <t>Diamondbacks</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr">
+      <c r="C37" t="inlineStr">
         <is>
           <t>Single-A California League</t>
         </is>
       </c>
-      <c r="D36" t="inlineStr">
+      <c r="D37" t="inlineStr">
         <is>
           <t>Visalia Rawhide</t>
         </is>
       </c>
-      <c r="E36" t="inlineStr">
+      <c r="E37" t="inlineStr">
         <is>
           <t>C</t>
-        </is>
-      </c>
-      <c r="F36" t="inlineStr"/>
-    </row>
-    <row r="37">
-      <c r="A37" s="3" t="inlineStr">
-        <is>
-          <t>Hicklen, Brewer</t>
-        </is>
-      </c>
-      <c r="B37" s="3" t="inlineStr">
-        <is>
-          <t>Braves</t>
-        </is>
-      </c>
-      <c r="C37" s="3" t="inlineStr">
-        <is>
-          <t>Triple-A International League</t>
-        </is>
-      </c>
-      <c r="D37" s="3" t="inlineStr">
-        <is>
-          <t>Gwinnett Stripers</t>
-        </is>
-      </c>
-      <c r="E37" s="3" t="inlineStr">
-        <is>
-          <t>OF</t>
-        </is>
-      </c>
-      <c r="F37" s="3" t="inlineStr">
-        <is>
-          <t>TJ</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="3" t="inlineStr">
         <is>
-          <t>Hill, GJ</t>
+          <t>Hicklen, Brewer</t>
         </is>
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>Rockies</t>
+          <t>Braves</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t>Double-A Eastern League</t>
+          <t>Triple-A International League</t>
         </is>
       </c>
       <c r="D38" s="3" t="inlineStr">
         <is>
-          <t>Hartford Yard Goats</t>
+          <t>Gwinnett Stripers</t>
         </is>
       </c>
       <c r="E38" s="3" t="inlineStr">
         <is>
-          <t>INF</t>
+          <t>OF</t>
         </is>
       </c>
       <c r="F38" s="3" t="inlineStr">
         <is>
-          <t>AK</t>
+          <t>TJ</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
         <is>
-          <t>Hoerner, Nico</t>
+          <t>Hill, GJ</t>
         </is>
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>Cubs</t>
+          <t>Rockies</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>Major Leagues</t>
+          <t>Double-A Eastern League</t>
+        </is>
+      </c>
+      <c r="D39" s="3" t="inlineStr">
+        <is>
+          <t>Hartford Yard Goats</t>
         </is>
       </c>
       <c r="E39" s="3" t="inlineStr">
         <is>
-          <t>2B</t>
+          <t>INF</t>
         </is>
       </c>
       <c r="F39" s="3" t="inlineStr">
@@ -1660,22 +1664,22 @@
     <row r="40">
       <c r="A40" s="3" t="inlineStr">
         <is>
-          <t>Howard, Spencer</t>
+          <t>Hoerner, Nico</t>
         </is>
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>Yomiuri</t>
+          <t>Cubs</t>
         </is>
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>NPB</t>
+          <t>Major Leagues</t>
         </is>
       </c>
       <c r="E40" s="3" t="inlineStr">
         <is>
-          <t>RHP</t>
+          <t>2B</t>
         </is>
       </c>
       <c r="F40" s="3" t="inlineStr">
@@ -1687,22 +1691,17 @@
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
         <is>
-          <t>Hurd, Thatcher</t>
+          <t>Howard, Spencer</t>
         </is>
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>Yankees</t>
+          <t>Yomiuri</t>
         </is>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>R Florida Complex League</t>
-        </is>
-      </c>
-      <c r="D41" s="3" t="inlineStr">
-        <is>
-          <t>FCL Yankees</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E41" s="3" t="inlineStr">
@@ -1719,27 +1718,27 @@
     <row r="42">
       <c r="A42" s="3" t="inlineStr">
         <is>
-          <t>Ibarra, Ruben</t>
+          <t>Hurd, Thatcher</t>
         </is>
       </c>
       <c r="B42" s="3" t="inlineStr">
         <is>
-          <t>Reds</t>
+          <t>Yankees</t>
         </is>
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
-          <t>Double-A Southern League</t>
+          <t>R Florida Complex League</t>
         </is>
       </c>
       <c r="D42" s="3" t="inlineStr">
         <is>
-          <t>Chattanooga Lookouts</t>
+          <t>FCL Yankees</t>
         </is>
       </c>
       <c r="E42" s="3" t="inlineStr">
         <is>
-          <t>1B</t>
+          <t>RHP</t>
         </is>
       </c>
       <c r="F42" s="3" t="inlineStr">
@@ -1751,44 +1750,44 @@
     <row r="43">
       <c r="A43" s="3" t="inlineStr">
         <is>
-          <t>Johnson, Seth</t>
+          <t>Ibarra, Ruben</t>
         </is>
       </c>
       <c r="B43" s="3" t="inlineStr">
         <is>
-          <t>Phillies</t>
+          <t>Reds</t>
         </is>
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>Triple-A International League</t>
+          <t>Double-A Southern League</t>
         </is>
       </c>
       <c r="D43" s="3" t="inlineStr">
         <is>
-          <t>Lehigh Valley IronPigs</t>
+          <t>Chattanooga Lookouts</t>
         </is>
       </c>
       <c r="E43" s="3" t="inlineStr">
         <is>
-          <t>RHP</t>
+          <t>1B</t>
         </is>
       </c>
       <c r="F43" s="3" t="inlineStr">
         <is>
-          <t>JF</t>
+          <t>AK</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="3" t="inlineStr">
         <is>
-          <t>Juenger, Hayden</t>
+          <t>Johnson, Seth</t>
         </is>
       </c>
       <c r="B44" s="3" t="inlineStr">
         <is>
-          <t>Blue Jays</t>
+          <t>Phillies</t>
         </is>
       </c>
       <c r="C44" s="3" t="inlineStr">
@@ -1798,7 +1797,7 @@
       </c>
       <c r="D44" s="3" t="inlineStr">
         <is>
-          <t>Buffalo Bisons</t>
+          <t>Lehigh Valley IronPigs</t>
         </is>
       </c>
       <c r="E44" s="3" t="inlineStr">
@@ -1815,39 +1814,44 @@
     <row r="45">
       <c r="A45" s="3" t="inlineStr">
         <is>
-          <t>Keaschall, Luke</t>
+          <t>Juenger, Hayden</t>
         </is>
       </c>
       <c r="B45" s="3" t="inlineStr">
         <is>
-          <t>Twins</t>
+          <t>Blue Jays</t>
         </is>
       </c>
       <c r="C45" s="3" t="inlineStr">
         <is>
-          <t>Major Leagues</t>
+          <t>Triple-A International League</t>
+        </is>
+      </c>
+      <c r="D45" s="3" t="inlineStr">
+        <is>
+          <t>Buffalo Bisons</t>
         </is>
       </c>
       <c r="E45" s="3" t="inlineStr">
         <is>
-          <t>2B</t>
+          <t>RHP</t>
         </is>
       </c>
       <c r="F45" s="3" t="inlineStr">
         <is>
-          <t>AK</t>
+          <t>JF</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="3" t="inlineStr">
         <is>
-          <t>Kelly, Merrill</t>
+          <t>Keaschall, Luke</t>
         </is>
       </c>
       <c r="B46" s="3" t="inlineStr">
         <is>
-          <t>Diamondbacks</t>
+          <t>Twins</t>
         </is>
       </c>
       <c r="C46" s="3" t="inlineStr">
@@ -1857,7 +1861,7 @@
       </c>
       <c r="E46" s="3" t="inlineStr">
         <is>
-          <t>RHP</t>
+          <t>2B</t>
         </is>
       </c>
       <c r="F46" s="3" t="inlineStr">
@@ -1869,86 +1873,86 @@
     <row r="47">
       <c r="A47" s="3" t="inlineStr">
         <is>
-          <t>Klein, Matt</t>
+          <t>Kelly, Merrill</t>
         </is>
       </c>
       <c r="B47" s="3" t="inlineStr">
         <is>
-          <t>Rockies</t>
+          <t>Diamondbacks</t>
         </is>
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>Single-A California League</t>
-        </is>
-      </c>
-      <c r="D47" s="3" t="inlineStr">
-        <is>
-          <t>Fresno Grizzlies</t>
+          <t>Major Leagues</t>
         </is>
       </c>
       <c r="E47" s="3" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>RHP</t>
         </is>
       </c>
       <c r="F47" s="3" t="inlineStr">
         <is>
-          <t>JF</t>
+          <t>AK</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="3" t="inlineStr">
         <is>
-          <t>Krook, Matt</t>
+          <t>Klein, Matt</t>
         </is>
       </c>
       <c r="B48" s="3" t="inlineStr">
         <is>
-          <t>Athletics</t>
+          <t>Rockies</t>
         </is>
       </c>
       <c r="C48" s="3" t="inlineStr">
         <is>
-          <t>Triple-A Pacific Coast League</t>
+          <t>Single-A California League</t>
         </is>
       </c>
       <c r="D48" s="3" t="inlineStr">
         <is>
-          <t>Las Vegas Aviators</t>
+          <t>Fresno Grizzlies</t>
         </is>
       </c>
       <c r="E48" s="3" t="inlineStr">
         <is>
-          <t>LHP</t>
+          <t>C</t>
         </is>
       </c>
       <c r="F48" s="3" t="inlineStr">
         <is>
-          <t>AK</t>
+          <t>JF</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="3" t="inlineStr">
         <is>
-          <t>Lee, Brooks</t>
+          <t>Krook, Matt</t>
         </is>
       </c>
       <c r="B49" s="3" t="inlineStr">
         <is>
-          <t>Twins</t>
+          <t>Athletics</t>
         </is>
       </c>
       <c r="C49" s="3" t="inlineStr">
         <is>
-          <t>Major Leagues</t>
+          <t>Triple-A Pacific Coast League</t>
+        </is>
+      </c>
+      <c r="D49" s="3" t="inlineStr">
+        <is>
+          <t>Las Vegas Aviators</t>
         </is>
       </c>
       <c r="E49" s="3" t="inlineStr">
         <is>
-          <t>INF</t>
+          <t>LHP</t>
         </is>
       </c>
       <c r="F49" s="3" t="inlineStr">
@@ -1960,113 +1964,108 @@
     <row r="50">
       <c r="A50" s="3" t="inlineStr">
         <is>
-          <t>Mathison, Carter</t>
+          <t>Lee, Brooks</t>
         </is>
       </c>
       <c r="B50" s="3" t="inlineStr">
         <is>
-          <t>Phillies</t>
+          <t>Twins</t>
         </is>
       </c>
       <c r="C50" s="3" t="inlineStr">
         <is>
-          <t>High-A South Atlantic League</t>
-        </is>
-      </c>
-      <c r="D50" s="3" t="inlineStr">
-        <is>
-          <t>Jersey Shore BlueClaws</t>
+          <t>Major Leagues</t>
         </is>
       </c>
       <c r="E50" s="3" t="inlineStr">
         <is>
-          <t>OF</t>
+          <t>INF</t>
         </is>
       </c>
       <c r="F50" s="3" t="inlineStr">
         <is>
-          <t>JF</t>
+          <t>AK</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="3" t="inlineStr">
         <is>
-          <t>Mayer, Gunner</t>
+          <t>Mathison, Carter</t>
         </is>
       </c>
       <c r="B51" s="3" t="inlineStr">
         <is>
-          <t>Mariners</t>
+          <t>Phillies</t>
         </is>
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>Double-A Texas League</t>
+          <t>High-A South Atlantic League</t>
         </is>
       </c>
       <c r="D51" s="3" t="inlineStr">
         <is>
-          <t>Arkansas Travelers</t>
+          <t>Jersey Shore BlueClaws</t>
         </is>
       </c>
       <c r="E51" s="3" t="inlineStr">
         <is>
-          <t>RHP</t>
+          <t>OF</t>
         </is>
       </c>
       <c r="F51" s="3" t="inlineStr">
         <is>
-          <t>AK</t>
+          <t>JF</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="3" t="inlineStr">
         <is>
-          <t>McGuire, Reese</t>
+          <t>Mayer, Gunner</t>
         </is>
       </c>
       <c r="B52" s="3" t="inlineStr">
         <is>
-          <t>White Sox</t>
+          <t>Mariners</t>
         </is>
       </c>
       <c r="C52" s="3" t="inlineStr">
         <is>
-          <t>Major Leagues</t>
+          <t>Double-A Texas League</t>
+        </is>
+      </c>
+      <c r="D52" s="3" t="inlineStr">
+        <is>
+          <t>Arkansas Travelers</t>
         </is>
       </c>
       <c r="E52" s="3" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>RHP</t>
         </is>
       </c>
       <c r="F52" s="3" t="inlineStr">
         <is>
-          <t>TJ</t>
+          <t>AK</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="3" t="inlineStr">
         <is>
-          <t>McGuire, Shane</t>
+          <t>McGuire, Reese</t>
         </is>
       </c>
       <c r="B53" s="3" t="inlineStr">
         <is>
-          <t>Athletics</t>
+          <t>White Sox</t>
         </is>
       </c>
       <c r="C53" s="3" t="inlineStr">
         <is>
-          <t>Double-A Texas League</t>
-        </is>
-      </c>
-      <c r="D53" s="3" t="inlineStr">
-        <is>
-          <t>Midland RockHounds</t>
+          <t>Major Leagues</t>
         </is>
       </c>
       <c r="E53" s="3" t="inlineStr">
@@ -2083,39 +2082,39 @@
     <row r="54">
       <c r="A54" s="3" t="inlineStr">
         <is>
-          <t>Millar, Cam</t>
+          <t>McGuire, Shane</t>
         </is>
       </c>
       <c r="B54" s="3" t="inlineStr">
         <is>
-          <t>Royals</t>
+          <t>Athletics</t>
         </is>
       </c>
       <c r="C54" s="3" t="inlineStr">
         <is>
-          <t>R Arizona Complex League</t>
+          <t>Double-A Texas League</t>
         </is>
       </c>
       <c r="D54" s="3" t="inlineStr">
         <is>
-          <t>ACL Royals</t>
+          <t>Midland RockHounds</t>
         </is>
       </c>
       <c r="E54" s="3" t="inlineStr">
         <is>
-          <t>RHP</t>
+          <t>C</t>
         </is>
       </c>
       <c r="F54" s="3" t="inlineStr">
         <is>
-          <t>AK</t>
+          <t>TJ</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="3" t="inlineStr">
         <is>
-          <t>Monke, Caden</t>
+          <t>Millar, Cam</t>
         </is>
       </c>
       <c r="B55" s="3" t="inlineStr">
@@ -2125,115 +2124,130 @@
       </c>
       <c r="C55" s="3" t="inlineStr">
         <is>
-          <t>Double-A Texas League</t>
+          <t>R Arizona Complex League</t>
         </is>
       </c>
       <c r="D55" s="3" t="inlineStr">
         <is>
-          <t>NW Arkansas Naturals</t>
+          <t>ACL Royals</t>
         </is>
       </c>
       <c r="E55" s="3" t="inlineStr">
         <is>
-          <t>LHP</t>
+          <t>RHP</t>
         </is>
       </c>
       <c r="F55" s="3" t="inlineStr">
         <is>
-          <t>JF</t>
+          <t>AK</t>
         </is>
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="3" t="inlineStr">
-        <is>
-          <t>Moore, Grayson</t>
-        </is>
-      </c>
-      <c r="B56" s="3" t="inlineStr">
-        <is>
-          <t>Cubs</t>
-        </is>
-      </c>
-      <c r="C56" s="3" t="inlineStr">
-        <is>
-          <t>High-A Midwest League</t>
-        </is>
-      </c>
-      <c r="D56" s="3" t="inlineStr">
-        <is>
-          <t>South Bend Cubs</t>
-        </is>
-      </c>
-      <c r="E56" s="3" t="inlineStr">
-        <is>
-          <t>RHP</t>
-        </is>
-      </c>
-      <c r="F56" s="3" t="inlineStr">
-        <is>
-          <t>JF</t>
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Molony, Maddox</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Tigers</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Single-A Florida State League</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Lakeland Flying Tigers</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>SS</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>PC</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="3" t="inlineStr">
         <is>
-          <t>Mountcastle, Ryan</t>
+          <t>Monke, Caden</t>
         </is>
       </c>
       <c r="B57" s="3" t="inlineStr">
         <is>
-          <t>Orioles</t>
+          <t>Royals</t>
         </is>
       </c>
       <c r="C57" s="3" t="inlineStr">
         <is>
-          <t>Major Leagues</t>
+          <t>Double-A Texas League</t>
+        </is>
+      </c>
+      <c r="D57" s="3" t="inlineStr">
+        <is>
+          <t>NW Arkansas Naturals</t>
         </is>
       </c>
       <c r="E57" s="3" t="inlineStr">
         <is>
-          <t>1B</t>
+          <t>LHP</t>
         </is>
       </c>
       <c r="F57" s="3" t="inlineStr">
         <is>
-          <t>TJ</t>
+          <t>JF</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="3" t="inlineStr">
         <is>
-          <t>Murray, Tanner</t>
+          <t>Moore, Grayson</t>
         </is>
       </c>
       <c r="B58" s="3" t="inlineStr">
         <is>
-          <t>White Sox</t>
+          <t>Cubs</t>
+        </is>
+      </c>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>High-A Midwest League</t>
+        </is>
+      </c>
+      <c r="D58" s="3" t="inlineStr">
+        <is>
+          <t>South Bend Cubs</t>
         </is>
       </c>
       <c r="E58" s="3" t="inlineStr">
         <is>
-          <t>INF / OF</t>
+          <t>RHP</t>
         </is>
       </c>
       <c r="F58" s="3" t="inlineStr">
         <is>
-          <t>AK</t>
+          <t>JF</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="3" t="inlineStr">
         <is>
-          <t>Outman, James</t>
+          <t>Mountcastle, Ryan</t>
         </is>
       </c>
       <c r="B59" s="3" t="inlineStr">
         <is>
-          <t>Twins</t>
+          <t>Orioles</t>
         </is>
       </c>
       <c r="C59" s="3" t="inlineStr">
@@ -2243,66 +2257,51 @@
       </c>
       <c r="E59" s="3" t="inlineStr">
         <is>
-          <t>OF</t>
+          <t>1B</t>
         </is>
       </c>
       <c r="F59" s="3" t="inlineStr">
         <is>
-          <t>AK</t>
+          <t>TJ</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="3" t="inlineStr">
         <is>
-          <t>Palmquist, Carson</t>
+          <t>Murray, Tanner</t>
         </is>
       </c>
       <c r="B60" s="3" t="inlineStr">
         <is>
-          <t>Rockies</t>
-        </is>
-      </c>
-      <c r="C60" s="3" t="inlineStr">
-        <is>
-          <t>Triple-A Pacific Coast League</t>
-        </is>
-      </c>
-      <c r="D60" s="3" t="inlineStr">
-        <is>
-          <t>Albuquerque Isotopes</t>
+          <t>White Sox</t>
         </is>
       </c>
       <c r="E60" s="3" t="inlineStr">
         <is>
-          <t>LHP</t>
+          <t>INF / OF</t>
         </is>
       </c>
       <c r="F60" s="3" t="inlineStr">
         <is>
-          <t>TJ</t>
+          <t>AK</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="3" t="inlineStr">
         <is>
-          <t>Park, Eddie</t>
+          <t>Outman, James</t>
         </is>
       </c>
       <c r="B61" s="3" t="inlineStr">
         <is>
-          <t>White Sox</t>
+          <t>Twins</t>
         </is>
       </c>
       <c r="C61" s="3" t="inlineStr">
         <is>
-          <t>R Arizona Complex League</t>
-        </is>
-      </c>
-      <c r="D61" s="3" t="inlineStr">
-        <is>
-          <t>ACL White Sox</t>
+          <t>Major Leagues</t>
         </is>
       </c>
       <c r="E61" s="3" t="inlineStr">
@@ -2319,27 +2318,27 @@
     <row r="62">
       <c r="A62" s="3" t="inlineStr">
         <is>
-          <t>Petry, Ethan</t>
+          <t>Palmquist, Carson</t>
         </is>
       </c>
       <c r="B62" s="3" t="inlineStr">
         <is>
-          <t>Nationals</t>
+          <t>Rockies</t>
         </is>
       </c>
       <c r="C62" s="3" t="inlineStr">
         <is>
-          <t>High-A South Atlantic League</t>
+          <t>Triple-A Pacific Coast League</t>
         </is>
       </c>
       <c r="D62" s="3" t="inlineStr">
         <is>
-          <t>Wilmington Blue Rocks</t>
+          <t>Albuquerque Isotopes</t>
         </is>
       </c>
       <c r="E62" s="3" t="inlineStr">
         <is>
-          <t>3B</t>
+          <t>LHP</t>
         </is>
       </c>
       <c r="F62" s="3" t="inlineStr">
@@ -2351,12 +2350,12 @@
     <row r="63">
       <c r="A63" s="3" t="inlineStr">
         <is>
-          <t>Phillips, Evan</t>
+          <t>Park, Eddie</t>
         </is>
       </c>
       <c r="B63" s="3" t="inlineStr">
         <is>
-          <t>Dodgers</t>
+          <t>White Sox</t>
         </is>
       </c>
       <c r="C63" s="3" t="inlineStr">
@@ -2366,12 +2365,12 @@
       </c>
       <c r="D63" s="3" t="inlineStr">
         <is>
-          <t>ACL Dodgers</t>
+          <t>ACL White Sox</t>
         </is>
       </c>
       <c r="E63" s="3" t="inlineStr">
         <is>
-          <t>RHP</t>
+          <t>OF</t>
         </is>
       </c>
       <c r="F63" s="3" t="inlineStr">
@@ -2383,54 +2382,54 @@
     <row r="64">
       <c r="A64" s="3" t="inlineStr">
         <is>
-          <t>Reid, Dom</t>
+          <t>Petry, Ethan</t>
         </is>
       </c>
       <c r="B64" s="3" t="inlineStr">
         <is>
-          <t>Cubs</t>
+          <t>Nationals</t>
         </is>
       </c>
       <c r="C64" s="3" t="inlineStr">
         <is>
-          <t>Single-A Carolina League</t>
+          <t>High-A South Atlantic League</t>
         </is>
       </c>
       <c r="D64" s="3" t="inlineStr">
         <is>
-          <t>Myrtle Beach Pelicans</t>
+          <t>Wilmington Blue Rocks</t>
         </is>
       </c>
       <c r="E64" s="3" t="inlineStr">
         <is>
-          <t>RHP</t>
+          <t>3B</t>
         </is>
       </c>
       <c r="F64" s="3" t="inlineStr">
         <is>
-          <t>JF</t>
+          <t>TJ</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="3" t="inlineStr">
         <is>
-          <t>Richards, Trevor</t>
+          <t>Phillips, Evan</t>
         </is>
       </c>
       <c r="B65" s="3" t="inlineStr">
         <is>
-          <t>Phillies</t>
+          <t>Dodgers</t>
         </is>
       </c>
       <c r="C65" s="3" t="inlineStr">
         <is>
-          <t>Triple-A International League</t>
+          <t>R Arizona Complex League</t>
         </is>
       </c>
       <c r="D65" s="3" t="inlineStr">
         <is>
-          <t>Lehigh Valley IronPigs</t>
+          <t>ACL Dodgers</t>
         </is>
       </c>
       <c r="E65" s="3" t="inlineStr">
@@ -2440,125 +2439,125 @@
       </c>
       <c r="F65" s="3" t="inlineStr">
         <is>
-          <t>PC</t>
+          <t>AK</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="3" t="inlineStr">
         <is>
-          <t>Rios, Alberto</t>
+          <t>Reid, Dom</t>
         </is>
       </c>
       <c r="B66" s="3" t="inlineStr">
         <is>
-          <t>Angels</t>
+          <t>Cubs</t>
         </is>
       </c>
       <c r="C66" s="3" t="inlineStr">
         <is>
-          <t>R Arizona Complex League</t>
+          <t>Single-A Carolina League</t>
         </is>
       </c>
       <c r="D66" s="3" t="inlineStr">
         <is>
-          <t>ACL Angels</t>
+          <t>Myrtle Beach Pelicans</t>
         </is>
       </c>
       <c r="E66" s="3" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>RHP</t>
         </is>
       </c>
       <c r="F66" s="3" t="inlineStr">
         <is>
-          <t>AK</t>
+          <t>JF</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="3" t="inlineStr">
         <is>
-          <t>Rushing, Dalton</t>
+          <t>Richards, Trevor</t>
         </is>
       </c>
       <c r="B67" s="3" t="inlineStr">
         <is>
-          <t>Dodgers</t>
+          <t>Phillies</t>
         </is>
       </c>
       <c r="C67" s="3" t="inlineStr">
         <is>
-          <t>Major Leagues</t>
+          <t>Triple-A International League</t>
+        </is>
+      </c>
+      <c r="D67" s="3" t="inlineStr">
+        <is>
+          <t>Lehigh Valley IronPigs</t>
         </is>
       </c>
       <c r="E67" s="3" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>RHP</t>
         </is>
       </c>
       <c r="F67" s="3" t="inlineStr">
         <is>
-          <t>JF</t>
+          <t>PC</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="3" t="inlineStr">
         <is>
-          <t>Schweitzer, Tyler</t>
+          <t>Rios, Alberto</t>
         </is>
       </c>
       <c r="B68" s="3" t="inlineStr">
         <is>
-          <t>White Sox</t>
+          <t>Angels</t>
         </is>
       </c>
       <c r="C68" s="3" t="inlineStr">
         <is>
-          <t>Triple-A International League</t>
+          <t>R Arizona Complex League</t>
         </is>
       </c>
       <c r="D68" s="3" t="inlineStr">
         <is>
-          <t>Charlotte Knights</t>
+          <t>ACL Angels</t>
         </is>
       </c>
       <c r="E68" s="3" t="inlineStr">
         <is>
-          <t>LHP</t>
+          <t>C</t>
         </is>
       </c>
       <c r="F68" s="3" t="inlineStr">
         <is>
-          <t>JF</t>
+          <t>AK</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="3" t="inlineStr">
         <is>
-          <t>Short, Avery</t>
+          <t>Rushing, Dalton</t>
         </is>
       </c>
       <c r="B69" s="3" t="inlineStr">
         <is>
-          <t>Diamondbacks</t>
+          <t>Dodgers</t>
         </is>
       </c>
       <c r="C69" s="3" t="inlineStr">
         <is>
-          <t>Double-A Texas League</t>
-        </is>
-      </c>
-      <c r="D69" s="3" t="inlineStr">
-        <is>
-          <t>Amarillo Sod Poodles</t>
+          <t>Major Leagues</t>
         </is>
       </c>
       <c r="E69" s="3" t="inlineStr">
         <is>
-          <t>LHP</t>
+          <t>C</t>
         </is>
       </c>
       <c r="F69" s="3" t="inlineStr">
@@ -2570,22 +2569,27 @@
     <row r="70">
       <c r="A70" s="3" t="inlineStr">
         <is>
-          <t>Smith, Will</t>
+          <t>Schweitzer, Tyler</t>
         </is>
       </c>
       <c r="B70" s="3" t="inlineStr">
         <is>
-          <t>Dodgers</t>
+          <t>White Sox</t>
         </is>
       </c>
       <c r="C70" s="3" t="inlineStr">
         <is>
-          <t>Major Leagues</t>
+          <t>Triple-A International League</t>
+        </is>
+      </c>
+      <c r="D70" s="3" t="inlineStr">
+        <is>
+          <t>Charlotte Knights</t>
         </is>
       </c>
       <c r="E70" s="3" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>LHP</t>
         </is>
       </c>
       <c r="F70" s="3" t="inlineStr">
@@ -2597,54 +2601,49 @@
     <row r="71">
       <c r="A71" s="3" t="inlineStr">
         <is>
-          <t>Song, Noah</t>
+          <t>Short, Avery</t>
         </is>
       </c>
       <c r="B71" s="3" t="inlineStr">
         <is>
-          <t>Red Sox</t>
+          <t>Diamondbacks</t>
         </is>
       </c>
       <c r="C71" s="3" t="inlineStr">
         <is>
-          <t>Triple-A International League</t>
+          <t>Double-A Texas League</t>
         </is>
       </c>
       <c r="D71" s="3" t="inlineStr">
         <is>
-          <t>Worcester Red Sox</t>
+          <t>Amarillo Sod Poodles</t>
         </is>
       </c>
       <c r="E71" s="3" t="inlineStr">
         <is>
-          <t>RHP</t>
+          <t>LHP</t>
         </is>
       </c>
       <c r="F71" s="3" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>JF</t>
         </is>
       </c>
     </row>
     <row r="72" customFormat="1" s="4">
       <c r="A72" s="3" t="inlineStr">
         <is>
-          <t>Stafford, Ryan</t>
+          <t>Smith, Will</t>
         </is>
       </c>
       <c r="B72" s="3" t="inlineStr">
         <is>
-          <t>Orioles</t>
+          <t>Dodgers</t>
         </is>
       </c>
       <c r="C72" s="3" t="inlineStr">
         <is>
-          <t>High-A South Atlantic League</t>
-        </is>
-      </c>
-      <c r="D72" s="3" t="inlineStr">
-        <is>
-          <t>Frederick Keys</t>
+          <t>Major Leagues</t>
         </is>
       </c>
       <c r="E72" s="3" t="inlineStr">
@@ -2654,107 +2653,107 @@
       </c>
       <c r="F72" s="3" t="inlineStr">
         <is>
-          <t>AK</t>
+          <t>JF</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="3" t="inlineStr">
         <is>
-          <t>Stanavich, Dale</t>
+          <t>Song, Noah</t>
         </is>
       </c>
       <c r="B73" s="3" t="inlineStr">
         <is>
-          <t>Giants</t>
-        </is>
-      </c>
-      <c r="C73" s="3" t="n"/>
-      <c r="D73" s="3" t="n"/>
+          <t>Red Sox</t>
+        </is>
+      </c>
+      <c r="C73" s="3" t="inlineStr">
+        <is>
+          <t>Triple-A International League</t>
+        </is>
+      </c>
+      <c r="D73" s="3" t="inlineStr">
+        <is>
+          <t>Worcester Red Sox</t>
+        </is>
+      </c>
       <c r="E73" s="3" t="inlineStr">
         <is>
-          <t>LHP</t>
+          <t>RHP</t>
         </is>
       </c>
       <c r="F73" s="3" t="inlineStr">
         <is>
-          <t>TJ</t>
+          <t>S</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="3" t="inlineStr">
         <is>
-          <t>Stephens, Jackson</t>
+          <t>Stafford, Ryan</t>
         </is>
       </c>
       <c r="B74" s="3" t="inlineStr">
         <is>
-          <t>Uni Lions (CPBL)</t>
+          <t>Orioles</t>
+        </is>
+      </c>
+      <c r="C74" s="3" t="inlineStr">
+        <is>
+          <t>High-A South Atlantic League</t>
+        </is>
+      </c>
+      <c r="D74" s="3" t="inlineStr">
+        <is>
+          <t>Frederick Keys</t>
         </is>
       </c>
       <c r="E74" s="3" t="inlineStr">
         <is>
-          <t>RHP</t>
+          <t>C</t>
         </is>
       </c>
       <c r="F74" s="3" t="inlineStr">
         <is>
-          <t>TJ</t>
+          <t>AK</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="3" t="inlineStr">
         <is>
-          <t>Stephenson, Robert</t>
+          <t>Stanavich, Dale</t>
         </is>
       </c>
       <c r="B75" s="3" t="inlineStr">
         <is>
-          <t>Angels</t>
-        </is>
-      </c>
-      <c r="C75" s="3" t="inlineStr">
-        <is>
-          <t>R Arizona Complex League</t>
-        </is>
-      </c>
-      <c r="D75" s="3" t="inlineStr">
-        <is>
-          <t>ACL Angels</t>
-        </is>
-      </c>
+          <t>Giants</t>
+        </is>
+      </c>
+      <c r="C75" s="3" t="n"/>
+      <c r="D75" s="3" t="n"/>
       <c r="E75" s="3" t="inlineStr">
         <is>
-          <t>RHP</t>
+          <t>LHP</t>
         </is>
       </c>
       <c r="F75" s="3" t="inlineStr">
         <is>
-          <t>AK</t>
+          <t>TJ</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="3" t="inlineStr">
         <is>
-          <t>Stuart, Tyler</t>
+          <t>Stephens, Jackson</t>
         </is>
       </c>
       <c r="B76" s="3" t="inlineStr">
         <is>
-          <t>Nationals</t>
-        </is>
-      </c>
-      <c r="C76" s="3" t="inlineStr">
-        <is>
-          <t>R Florida Complex League</t>
-        </is>
-      </c>
-      <c r="D76" s="3" t="inlineStr">
-        <is>
-          <t>FCL Nationals</t>
+          <t>Uni Lions (CPBL)</t>
         </is>
       </c>
       <c r="E76" s="3" t="inlineStr">
@@ -2764,56 +2763,61 @@
       </c>
       <c r="F76" s="3" t="inlineStr">
         <is>
-          <t>JF</t>
+          <t>TJ</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="3" t="inlineStr">
         <is>
-          <t>Sweeney, Trey</t>
+          <t>Stephenson, Robert</t>
         </is>
       </c>
       <c r="B77" s="3" t="inlineStr">
         <is>
-          <t>Tigers</t>
+          <t>Angels</t>
         </is>
       </c>
       <c r="C77" s="3" t="inlineStr">
         <is>
-          <t>Major Leagues</t>
+          <t>R Arizona Complex League</t>
+        </is>
+      </c>
+      <c r="D77" s="3" t="inlineStr">
+        <is>
+          <t>ACL Angels</t>
         </is>
       </c>
       <c r="E77" s="3" t="inlineStr">
         <is>
-          <t>SS</t>
+          <t>RHP</t>
         </is>
       </c>
       <c r="F77" s="3" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>AK</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="3" t="inlineStr">
         <is>
-          <t>Thorpe, Drew</t>
+          <t>Stuart, Tyler</t>
         </is>
       </c>
       <c r="B78" s="3" t="inlineStr">
         <is>
-          <t>White Sox</t>
+          <t>Nationals</t>
         </is>
       </c>
       <c r="C78" s="3" t="inlineStr">
         <is>
-          <t>R Arizona Complex League</t>
+          <t>R Florida Complex League</t>
         </is>
       </c>
       <c r="D78" s="3" t="inlineStr">
         <is>
-          <t>ACL White Sox</t>
+          <t>FCL Nationals</t>
         </is>
       </c>
       <c r="E78" s="3" t="inlineStr">
@@ -2823,56 +2827,56 @@
       </c>
       <c r="F78" s="3" t="inlineStr">
         <is>
-          <t>AK</t>
+          <t>JF</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="3" t="inlineStr">
         <is>
-          <t>Tookoian, Sam</t>
+          <t>Sweeney, Trey</t>
         </is>
       </c>
       <c r="B79" s="3" t="inlineStr">
         <is>
-          <t>Angels</t>
+          <t>Tigers</t>
         </is>
       </c>
       <c r="C79" s="3" t="inlineStr">
         <is>
-          <t>High-A Northwest League</t>
-        </is>
-      </c>
-      <c r="D79" s="3" t="inlineStr">
-        <is>
-          <t>Tri-City Dust Devils</t>
+          <t>Major Leagues</t>
         </is>
       </c>
       <c r="E79" s="3" t="inlineStr">
         <is>
-          <t>RHP</t>
+          <t>SS</t>
         </is>
       </c>
       <c r="F79" s="3" t="inlineStr">
         <is>
-          <t>AK</t>
+          <t>S</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="3" t="inlineStr">
         <is>
-          <t>Treinen, Blake</t>
+          <t>Thorpe, Drew</t>
         </is>
       </c>
       <c r="B80" s="3" t="inlineStr">
         <is>
-          <t>Dodgers</t>
+          <t>White Sox</t>
         </is>
       </c>
       <c r="C80" s="3" t="inlineStr">
         <is>
-          <t>Major Leagues</t>
+          <t>R Arizona Complex League</t>
+        </is>
+      </c>
+      <c r="D80" s="3" t="inlineStr">
+        <is>
+          <t>ACL White Sox</t>
         </is>
       </c>
       <c r="E80" s="3" t="inlineStr">
@@ -2889,27 +2893,27 @@
     <row r="81">
       <c r="A81" s="3" t="inlineStr">
         <is>
-          <t>Troy, Tommy</t>
+          <t>Tookoian, Sam</t>
         </is>
       </c>
       <c r="B81" s="3" t="inlineStr">
         <is>
-          <t>Diamondbacks</t>
+          <t>Angels</t>
         </is>
       </c>
       <c r="C81" s="3" t="inlineStr">
         <is>
-          <t>Triple-A Pacific Coast League</t>
+          <t>High-A Northwest League</t>
         </is>
       </c>
       <c r="D81" s="3" t="inlineStr">
         <is>
-          <t>Reno Aces</t>
+          <t>Tri-City Dust Devils</t>
         </is>
       </c>
       <c r="E81" s="3" t="inlineStr">
         <is>
-          <t>SS</t>
+          <t>RHP</t>
         </is>
       </c>
       <c r="F81" s="3" t="inlineStr">
@@ -2921,22 +2925,17 @@
     <row r="82">
       <c r="A82" s="3" t="inlineStr">
         <is>
-          <t>True, Derek</t>
+          <t>Treinen, Blake</t>
         </is>
       </c>
       <c r="B82" s="3" t="inlineStr">
         <is>
-          <t>Astros</t>
+          <t>Dodgers</t>
         </is>
       </c>
       <c r="C82" s="3" t="inlineStr">
         <is>
-          <t>Double-A Texas League</t>
-        </is>
-      </c>
-      <c r="D82" s="3" t="inlineStr">
-        <is>
-          <t>Corpus Christi Hooks</t>
+          <t>Major Leagues</t>
         </is>
       </c>
       <c r="E82" s="3" t="inlineStr">
@@ -2953,27 +2952,27 @@
     <row r="83">
       <c r="A83" s="3" t="inlineStr">
         <is>
-          <t>Vanderhei, Ryan</t>
+          <t>Troy, Tommy</t>
         </is>
       </c>
       <c r="B83" s="3" t="inlineStr">
         <is>
-          <t>Giants</t>
+          <t>Diamondbacks</t>
         </is>
       </c>
       <c r="C83" s="3" t="inlineStr">
         <is>
-          <t>High-A Northwest League</t>
+          <t>Triple-A Pacific Coast League</t>
         </is>
       </c>
       <c r="D83" s="3" t="inlineStr">
         <is>
-          <t>Eugene Emeralds</t>
+          <t>Reno Aces</t>
         </is>
       </c>
       <c r="E83" s="3" t="inlineStr">
         <is>
-          <t>RHP</t>
+          <t>SS</t>
         </is>
       </c>
       <c r="F83" s="3" t="inlineStr">
@@ -2985,17 +2984,22 @@
     <row r="84">
       <c r="A84" s="3" t="inlineStr">
         <is>
-          <t>Varland, Gus</t>
+          <t>True, Derek</t>
         </is>
       </c>
       <c r="B84" s="3" t="inlineStr">
         <is>
-          <t>Nationals</t>
+          <t>Astros</t>
         </is>
       </c>
       <c r="C84" s="3" t="inlineStr">
         <is>
-          <t>Major Leagues</t>
+          <t>Double-A Texas League</t>
+        </is>
+      </c>
+      <c r="D84" s="3" t="inlineStr">
+        <is>
+          <t>Corpus Christi Hooks</t>
         </is>
       </c>
       <c r="E84" s="3" t="inlineStr">
@@ -3012,34 +3016,39 @@
     <row r="85">
       <c r="A85" s="3" t="inlineStr">
         <is>
-          <t>Vierling, Matt</t>
+          <t>Vanderhei, Ryan</t>
         </is>
       </c>
       <c r="B85" s="3" t="inlineStr">
         <is>
-          <t>Tigers</t>
+          <t>Giants</t>
         </is>
       </c>
       <c r="C85" s="3" t="inlineStr">
         <is>
-          <t>Major Leagues</t>
+          <t>High-A Northwest League</t>
+        </is>
+      </c>
+      <c r="D85" s="3" t="inlineStr">
+        <is>
+          <t>Eugene Emeralds</t>
         </is>
       </c>
       <c r="E85" s="3" t="inlineStr">
         <is>
-          <t>OF</t>
+          <t>RHP</t>
         </is>
       </c>
       <c r="F85" s="3" t="inlineStr">
         <is>
-          <t>TJ</t>
+          <t>AK</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="3" t="inlineStr">
         <is>
-          <t>Waldichuk, Ken</t>
+          <t>Varland, Gus</t>
         </is>
       </c>
       <c r="B86" s="3" t="inlineStr">
@@ -3054,93 +3063,88 @@
       </c>
       <c r="E86" s="3" t="inlineStr">
         <is>
-          <t>LHP</t>
+          <t>RHP</t>
         </is>
       </c>
       <c r="F86" s="3" t="inlineStr">
         <is>
-          <t>PC</t>
+          <t>AK</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="3" t="inlineStr">
         <is>
-          <t>Warrecker, Bryce</t>
+          <t>Vierling, Matt</t>
         </is>
       </c>
       <c r="B87" s="3" t="inlineStr">
         <is>
-          <t>Yankees</t>
+          <t>Tigers</t>
         </is>
       </c>
       <c r="C87" s="3" t="inlineStr">
         <is>
-          <t>High-A South Atlantic League</t>
-        </is>
-      </c>
-      <c r="D87" s="3" t="inlineStr">
-        <is>
-          <t>Hudson Valley Renegades</t>
+          <t>Major Leagues</t>
         </is>
       </c>
       <c r="E87" s="3" t="inlineStr">
         <is>
-          <t>RHP</t>
+          <t>OF</t>
         </is>
       </c>
       <c r="F87" s="3" t="inlineStr">
         <is>
-          <t>AK</t>
+          <t>TJ</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="3" t="inlineStr">
         <is>
-          <t>Wheeler, Jack</t>
+          <t>Waldichuk, Ken</t>
         </is>
       </c>
       <c r="B88" s="3" t="inlineStr">
         <is>
-          <t>Rangers</t>
+          <t>Nationals</t>
         </is>
       </c>
       <c r="C88" s="3" t="inlineStr">
         <is>
-          <t>R Arizona Complex League</t>
-        </is>
-      </c>
-      <c r="D88" s="3" t="inlineStr">
-        <is>
-          <t>ACL Rangers</t>
+          <t>Major Leagues</t>
         </is>
       </c>
       <c r="E88" s="3" t="inlineStr">
         <is>
-          <t>3B</t>
+          <t>LHP</t>
         </is>
       </c>
       <c r="F88" s="3" t="inlineStr">
         <is>
-          <t>JF</t>
+          <t>PC</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="3" t="inlineStr">
         <is>
-          <t>White, Mitch</t>
+          <t>Warrecker, Bryce</t>
         </is>
       </c>
       <c r="B89" s="3" t="inlineStr">
         <is>
-          <t>SSG Landers</t>
+          <t>Yankees</t>
         </is>
       </c>
       <c r="C89" s="3" t="inlineStr">
         <is>
-          <t>KBO</t>
+          <t>High-A South Atlantic League</t>
+        </is>
+      </c>
+      <c r="D89" s="3" t="inlineStr">
+        <is>
+          <t>Hudson Valley Renegades</t>
         </is>
       </c>
       <c r="E89" s="3" t="inlineStr">
@@ -3157,22 +3161,22 @@
     <row r="90">
       <c r="A90" s="3" t="inlineStr">
         <is>
-          <t>Wilken, Brock</t>
+          <t>Wheeler, Jack</t>
         </is>
       </c>
       <c r="B90" s="3" t="inlineStr">
         <is>
-          <t>Brewers</t>
+          <t>Rangers</t>
         </is>
       </c>
       <c r="C90" s="3" t="inlineStr">
         <is>
-          <t>Triple-A International League</t>
+          <t>R Arizona Complex League</t>
         </is>
       </c>
       <c r="D90" s="3" t="inlineStr">
         <is>
-          <t>Nashville Sounds</t>
+          <t>ACL Rangers</t>
         </is>
       </c>
       <c r="E90" s="3" t="inlineStr">
@@ -3182,34 +3186,29 @@
       </c>
       <c r="F90" s="3" t="inlineStr">
         <is>
-          <t>TJ</t>
+          <t>JF</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="3" t="inlineStr">
         <is>
-          <t>Wisdom, Patrick</t>
+          <t>White, Mitch</t>
         </is>
       </c>
       <c r="B91" s="3" t="inlineStr">
         <is>
-          <t>Mariners</t>
+          <t>SSG Landers</t>
         </is>
       </c>
       <c r="C91" s="3" t="inlineStr">
         <is>
-          <t>Triple-A Pacific Coast League</t>
-        </is>
-      </c>
-      <c r="D91" s="3" t="inlineStr">
-        <is>
-          <t>Tacoma Rainiers</t>
+          <t>KBO</t>
         </is>
       </c>
       <c r="E91" s="3" t="inlineStr">
         <is>
-          <t>3B</t>
+          <t>RHP</t>
         </is>
       </c>
       <c r="F91" s="3" t="inlineStr">
@@ -3221,49 +3220,59 @@
     <row r="92">
       <c r="A92" s="3" t="inlineStr">
         <is>
-          <t>Woo, Bryan</t>
+          <t>Wilken, Brock</t>
         </is>
       </c>
       <c r="B92" s="3" t="inlineStr">
         <is>
-          <t>Mariners</t>
+          <t>Brewers</t>
         </is>
       </c>
       <c r="C92" s="3" t="inlineStr">
         <is>
-          <t>Major Leagues</t>
+          <t>Triple-A International League</t>
+        </is>
+      </c>
+      <c r="D92" s="3" t="inlineStr">
+        <is>
+          <t>Nashville Sounds</t>
         </is>
       </c>
       <c r="E92" s="3" t="inlineStr">
         <is>
-          <t>RHP</t>
+          <t>3B</t>
         </is>
       </c>
       <c r="F92" s="3" t="inlineStr">
         <is>
-          <t>AK</t>
+          <t>TJ</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="3" t="inlineStr">
         <is>
-          <t>Yorke, Nick</t>
+          <t>Wisdom, Patrick</t>
         </is>
       </c>
       <c r="B93" s="3" t="inlineStr">
         <is>
-          <t>Pirates</t>
+          <t>Mariners</t>
         </is>
       </c>
       <c r="C93" s="3" t="inlineStr">
         <is>
-          <t>Major Leagues</t>
+          <t>Triple-A Pacific Coast League</t>
+        </is>
+      </c>
+      <c r="D93" s="3" t="inlineStr">
+        <is>
+          <t>Tacoma Rainiers</t>
         </is>
       </c>
       <c r="E93" s="3" t="inlineStr">
         <is>
-          <t>2B</t>
+          <t>3B</t>
         </is>
       </c>
       <c r="F93" s="3" t="inlineStr">
@@ -3275,117 +3284,147 @@
     <row r="94">
       <c r="A94" s="3" t="inlineStr">
         <is>
+          <t>Woo, Bryan</t>
+        </is>
+      </c>
+      <c r="B94" s="3" t="inlineStr">
+        <is>
+          <t>Mariners</t>
+        </is>
+      </c>
+      <c r="C94" s="3" t="inlineStr">
+        <is>
+          <t>Major Leagues</t>
+        </is>
+      </c>
+      <c r="E94" s="3" t="inlineStr">
+        <is>
+          <t>RHP</t>
+        </is>
+      </c>
+      <c r="F94" s="3" t="inlineStr">
+        <is>
+          <t>AK</t>
+        </is>
+      </c>
+    </row>
+    <row r="95" ht="16" customFormat="1" customHeight="1" s="6" thickBot="1">
+      <c r="A95" s="3" t="inlineStr">
+        <is>
+          <t>Yorke, Nick</t>
+        </is>
+      </c>
+      <c r="B95" s="3" t="inlineStr">
+        <is>
+          <t>Pirates</t>
+        </is>
+      </c>
+      <c r="C95" s="3" t="inlineStr">
+        <is>
+          <t>Major Leagues</t>
+        </is>
+      </c>
+      <c r="E95" s="3" t="inlineStr">
+        <is>
+          <t>2B</t>
+        </is>
+      </c>
+      <c r="F95" s="3" t="inlineStr">
+        <is>
+          <t>AK</t>
+        </is>
+      </c>
+    </row>
+    <row r="96" ht="16" customFormat="1" customHeight="1" s="4" thickTop="1">
+      <c r="A96" s="3" t="inlineStr">
+        <is>
           <t>Zavala, Aaron</t>
         </is>
       </c>
-      <c r="B94" s="3" t="inlineStr">
+      <c r="B96" s="3" t="inlineStr">
         <is>
           <t>Rangers</t>
         </is>
       </c>
-      <c r="C94" s="3" t="inlineStr">
+      <c r="C96" s="3" t="inlineStr">
         <is>
           <t>Triple-A Pacific Coast League</t>
         </is>
       </c>
-      <c r="D94" s="3" t="inlineStr">
+      <c r="D96" s="3" t="inlineStr">
         <is>
           <t>Round Rock Express</t>
         </is>
       </c>
-      <c r="E94" s="3" t="inlineStr">
+      <c r="E96" s="3" t="inlineStr">
         <is>
           <t>OF</t>
         </is>
       </c>
-      <c r="F94" s="3" t="inlineStr">
-        <is>
-          <t>AK</t>
-        </is>
-      </c>
-    </row>
-    <row r="95" ht="16" customFormat="1" customHeight="1" s="6" thickBot="1">
-      <c r="A95" s="3" t="n"/>
-    </row>
-    <row r="96" ht="16" customFormat="1" customHeight="1" s="4" thickTop="1">
-      <c r="A96" s="5" t="inlineStr">
-        <is>
-          <t>Nakken, Alyssa</t>
-        </is>
-      </c>
-      <c r="B96" s="5" t="inlineStr">
-        <is>
-          <t>Guardians</t>
-        </is>
-      </c>
-      <c r="C96" s="5" t="n"/>
-      <c r="D96" s="5" t="n"/>
-      <c r="E96" s="5" t="n"/>
-      <c r="F96" s="5" t="n"/>
+      <c r="F96" s="3" t="inlineStr">
+        <is>
+          <t>AK</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="3" t="n"/>
-      <c r="B97" s="3" t="n"/>
-      <c r="C97" s="3" t="n"/>
-      <c r="D97" s="3" t="n"/>
-      <c r="E97" s="3" t="n"/>
-      <c r="F97" s="3" t="n"/>
     </row>
     <row r="98">
-      <c r="A98" s="3" t="inlineStr">
-        <is>
-          <t>Alexander, Scott</t>
-        </is>
-      </c>
-      <c r="B98" s="3" t="inlineStr">
-        <is>
-          <t>Free Agent</t>
-        </is>
-      </c>
-      <c r="E98" s="3" t="inlineStr">
-        <is>
-          <t>LHP</t>
-        </is>
-      </c>
+      <c r="A98" s="5" t="inlineStr">
+        <is>
+          <t>Nakken, Alyssa</t>
+        </is>
+      </c>
+      <c r="B98" s="5" t="inlineStr">
+        <is>
+          <t>Guardians</t>
+        </is>
+      </c>
+      <c r="C98" s="5" t="n"/>
+      <c r="D98" s="5" t="n"/>
+      <c r="E98" s="5" t="n"/>
+      <c r="F98" s="5" t="n"/>
     </row>
     <row r="99">
-      <c r="A99" s="3" t="inlineStr">
-        <is>
-          <t>Barber, Colin</t>
-        </is>
-      </c>
-      <c r="B99" s="3" t="inlineStr">
-        <is>
-          <t>Free Agent</t>
-        </is>
-      </c>
-      <c r="E99" s="3" t="inlineStr">
-        <is>
-          <t>OF</t>
-        </is>
-      </c>
+      <c r="A99" s="3" t="n"/>
+      <c r="B99" s="3" t="n"/>
+      <c r="C99" s="3" t="n"/>
+      <c r="D99" s="3" t="n"/>
+      <c r="E99" s="3" t="n"/>
+      <c r="F99" s="3" t="n"/>
     </row>
     <row r="100">
       <c r="A100" s="3" t="inlineStr">
         <is>
-          <t>Boyer, Logan</t>
+          <t>Alexander, Scott</t>
         </is>
       </c>
       <c r="B100" s="3" t="inlineStr">
         <is>
-          <t>Free Agent</t>
+          <t>Royals</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>Triple-A International League</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>Omaha Storm Chasers</t>
         </is>
       </c>
       <c r="E100" s="3" t="inlineStr">
         <is>
-          <t>RHP</t>
+          <t>LHP</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="3" t="inlineStr">
         <is>
-          <t>Dipoto, Jonah</t>
+          <t>Barber, Colin</t>
         </is>
       </c>
       <c r="B101" s="3" t="inlineStr">
@@ -3395,14 +3434,14 @@
       </c>
       <c r="E101" s="3" t="inlineStr">
         <is>
-          <t>RHP</t>
+          <t>OF</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="3" t="inlineStr">
         <is>
-          <t>Jefferies, Daulton</t>
+          <t>Boyer, Logan</t>
         </is>
       </c>
       <c r="B102" s="3" t="inlineStr">
@@ -3419,7 +3458,7 @@
     <row r="103">
       <c r="A103" s="3" t="inlineStr">
         <is>
-          <t>Puckett, AJ</t>
+          <t>Dipoto, Jonah</t>
         </is>
       </c>
       <c r="B103" s="3" t="inlineStr">
@@ -3436,7 +3475,7 @@
     <row r="104">
       <c r="A104" s="3" t="inlineStr">
         <is>
-          <t>Sampson, Adrian</t>
+          <t>Jefferies, Daulton</t>
         </is>
       </c>
       <c r="B104" s="3" t="inlineStr">
@@ -3453,7 +3492,7 @@
     <row r="105">
       <c r="A105" s="3" t="inlineStr">
         <is>
-          <t>Viars, Jordan</t>
+          <t>Puckett, AJ</t>
         </is>
       </c>
       <c r="B105" s="3" t="inlineStr">
@@ -3463,32 +3502,60 @@
       </c>
       <c r="E105" s="3" t="inlineStr">
         <is>
-          <t>OF</t>
+          <t>RHP</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="3" t="inlineStr">
         <is>
+          <t>Sampson, Adrian</t>
+        </is>
+      </c>
+      <c r="B106" s="3" t="inlineStr">
+        <is>
+          <t>Free Agent</t>
+        </is>
+      </c>
+      <c r="E106" s="3" t="inlineStr">
+        <is>
+          <t>RHP</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="3" t="inlineStr">
+        <is>
+          <t>Viars, Jordan</t>
+        </is>
+      </c>
+      <c r="B107" s="3" t="inlineStr">
+        <is>
+          <t>Free Agent</t>
+        </is>
+      </c>
+      <c r="E107" s="3" t="inlineStr">
+        <is>
+          <t>OF</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="3" t="inlineStr">
+        <is>
           <t>Wolf, Adam</t>
         </is>
       </c>
-      <c r="B106" s="3" t="inlineStr">
+      <c r="B108" s="3" t="inlineStr">
         <is>
           <t>Free Agent</t>
         </is>
       </c>
-      <c r="E106" s="3" t="inlineStr">
+      <c r="E108" s="3" t="inlineStr">
         <is>
           <t>LHP</t>
         </is>
       </c>
-    </row>
-    <row r="107">
-      <c r="A107" s="3" t="n"/>
-    </row>
-    <row r="108">
-      <c r="A108" s="3" t="n"/>
     </row>
     <row r="109">
       <c r="A109" s="3" t="n"/>
@@ -3519,6 +3586,12 @@
     </row>
     <row r="118">
       <c r="A118" s="3" t="n"/>
+    </row>
+    <row r="119">
+      <c r="A119" s="3" t="n"/>
+    </row>
+    <row r="120">
+      <c r="A120" s="3" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Set Scott Alexander to AK and Devin Bell to AR/AK on the tracker.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/client_lists/Client List - 04-15-26.xlsx
+++ b/client_lists/Client List - 04-15-26.xlsx
@@ -838,7 +838,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>AK</t>
+          <t>AR/AK</t>
         </is>
       </c>
     </row>
@@ -3420,6 +3420,11 @@
           <t>LHP</t>
         </is>
       </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>AK</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="3" t="inlineStr">

</xml_diff>